<commit_message>
added raw symbiont alignment; wgcna/table updates
</commit_message>
<xml_diff>
--- a/tables/Table S10.xlsx
+++ b/tables/Table S10.xlsx
@@ -608,7 +608,7 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>Bleaching vs OA</t>
+          <t>OA &amp; Bleaching</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
@@ -829,7 +829,7 @@
     <row r="10" s="6">
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>OA + Bleaching vs OA</t>
+          <t>OA &amp; OA + Bleaching</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Bleaching vs OA</t>
+          <t>OA &amp; Bleaching</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
@@ -1114,7 +1114,7 @@
     <row r="20" s="6">
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>OA + Bleaching vs OA</t>
+          <t>OA &amp; OA + Bleaching</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">

</xml_diff>